<commit_message>
feat: áreas, tarifas, roles por módulo y planos de reunión (v0.2.0)
</commit_message>
<xml_diff>
--- a/backend/templates/lots.xlsx
+++ b/backend/templates/lots.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lotes" sheetId="1" r:id="R632f75ebcc4a46cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R0505829339ec42aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lotes" sheetId="1" r:id="Ra70ec059cb7441fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R94ee14c2357b4ed9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
+    <x:numFmt numFmtId="202" formatCode="0.000000"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -74,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -82,6 +83,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -296,6 +298,9 @@
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -316,6 +321,15 @@
       </x:c>
       <x:c r="F1" s="3" t="str">
         <x:v>Estado</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Área m²</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Área vara²</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>Unidad de precio</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
@@ -325,6 +339,9 @@
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="5"/>
       <x:c r="F2" s="5"/>
+      <x:c r="G2" s="7"/>
+      <x:c r="H2" s="7"/>
+      <x:c r="I2" s="5"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="5"/>
@@ -333,6 +350,9 @@
       <x:c r="D3" s="6"/>
       <x:c r="E3" s="5"/>
       <x:c r="F3" s="5"/>
+      <x:c r="G3" s="7"/>
+      <x:c r="H3" s="7"/>
+      <x:c r="I3" s="5"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="5"/>
@@ -341,6 +361,9 @@
       <x:c r="D4" s="6"/>
       <x:c r="E4" s="5"/>
       <x:c r="F4" s="5"/>
+      <x:c r="G4" s="7"/>
+      <x:c r="H4" s="7"/>
+      <x:c r="I4" s="5"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="5"/>
@@ -349,6 +372,9 @@
       <x:c r="D5" s="6"/>
       <x:c r="E5" s="5"/>
       <x:c r="F5" s="5"/>
+      <x:c r="G5" s="7"/>
+      <x:c r="H5" s="7"/>
+      <x:c r="I5" s="5"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="5"/>
@@ -357,6 +383,9 @@
       <x:c r="D6" s="6"/>
       <x:c r="E6" s="5"/>
       <x:c r="F6" s="5"/>
+      <x:c r="G6" s="7"/>
+      <x:c r="H6" s="7"/>
+      <x:c r="I6" s="5"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="5"/>
@@ -365,6 +394,9 @@
       <x:c r="D7" s="6"/>
       <x:c r="E7" s="5"/>
       <x:c r="F7" s="5"/>
+      <x:c r="G7" s="7"/>
+      <x:c r="H7" s="7"/>
+      <x:c r="I7" s="5"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="5"/>
@@ -373,6 +405,9 @@
       <x:c r="D8" s="6"/>
       <x:c r="E8" s="5"/>
       <x:c r="F8" s="5"/>
+      <x:c r="G8" s="7"/>
+      <x:c r="H8" s="7"/>
+      <x:c r="I8" s="5"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="5"/>
@@ -381,6 +416,9 @@
       <x:c r="D9" s="6"/>
       <x:c r="E9" s="5"/>
       <x:c r="F9" s="5"/>
+      <x:c r="G9" s="7"/>
+      <x:c r="H9" s="7"/>
+      <x:c r="I9" s="5"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="5"/>
@@ -389,6 +427,9 @@
       <x:c r="D10" s="6"/>
       <x:c r="E10" s="5"/>
       <x:c r="F10" s="5"/>
+      <x:c r="G10" s="7"/>
+      <x:c r="H10" s="7"/>
+      <x:c r="I10" s="5"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="5"/>
@@ -397,6 +438,9 @@
       <x:c r="D11" s="6"/>
       <x:c r="E11" s="5"/>
       <x:c r="F11" s="5"/>
+      <x:c r="G11" s="7"/>
+      <x:c r="H11" s="7"/>
+      <x:c r="I11" s="5"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="5"/>
@@ -405,6 +449,9 @@
       <x:c r="D12" s="6"/>
       <x:c r="E12" s="5"/>
       <x:c r="F12" s="5"/>
+      <x:c r="G12" s="7"/>
+      <x:c r="H12" s="7"/>
+      <x:c r="I12" s="5"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="5"/>
@@ -413,6 +460,9 @@
       <x:c r="D13" s="6"/>
       <x:c r="E13" s="5"/>
       <x:c r="F13" s="5"/>
+      <x:c r="G13" s="7"/>
+      <x:c r="H13" s="7"/>
+      <x:c r="I13" s="5"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="5"/>
@@ -421,6 +471,9 @@
       <x:c r="D14" s="6"/>
       <x:c r="E14" s="5"/>
       <x:c r="F14" s="5"/>
+      <x:c r="G14" s="7"/>
+      <x:c r="H14" s="7"/>
+      <x:c r="I14" s="5"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="5"/>
@@ -429,6 +482,9 @@
       <x:c r="D15" s="6"/>
       <x:c r="E15" s="5"/>
       <x:c r="F15" s="5"/>
+      <x:c r="G15" s="7"/>
+      <x:c r="H15" s="7"/>
+      <x:c r="I15" s="5"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="5"/>
@@ -437,6 +493,9 @@
       <x:c r="D16" s="6"/>
       <x:c r="E16" s="5"/>
       <x:c r="F16" s="5"/>
+      <x:c r="G16" s="7"/>
+      <x:c r="H16" s="7"/>
+      <x:c r="I16" s="5"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="5"/>
@@ -445,6 +504,9 @@
       <x:c r="D17" s="6"/>
       <x:c r="E17" s="5"/>
       <x:c r="F17" s="5"/>
+      <x:c r="G17" s="7"/>
+      <x:c r="H17" s="7"/>
+      <x:c r="I17" s="5"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="5"/>
@@ -453,6 +515,9 @@
       <x:c r="D18" s="6"/>
       <x:c r="E18" s="5"/>
       <x:c r="F18" s="5"/>
+      <x:c r="G18" s="7"/>
+      <x:c r="H18" s="7"/>
+      <x:c r="I18" s="5"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="5"/>
@@ -461,6 +526,9 @@
       <x:c r="D19" s="6"/>
       <x:c r="E19" s="5"/>
       <x:c r="F19" s="5"/>
+      <x:c r="G19" s="7"/>
+      <x:c r="H19" s="7"/>
+      <x:c r="I19" s="5"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="5"/>
@@ -469,6 +537,9 @@
       <x:c r="D20" s="6"/>
       <x:c r="E20" s="5"/>
       <x:c r="F20" s="5"/>
+      <x:c r="G20" s="7"/>
+      <x:c r="H20" s="7"/>
+      <x:c r="I20" s="5"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="5"/>
@@ -477,6 +548,9 @@
       <x:c r="D21" s="6"/>
       <x:c r="E21" s="5"/>
       <x:c r="F21" s="5"/>
+      <x:c r="G21" s="7"/>
+      <x:c r="H21" s="7"/>
+      <x:c r="I21" s="5"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="5"/>
@@ -485,6 +559,9 @@
       <x:c r="D22" s="6"/>
       <x:c r="E22" s="5"/>
       <x:c r="F22" s="5"/>
+      <x:c r="G22" s="7"/>
+      <x:c r="H22" s="7"/>
+      <x:c r="I22" s="5"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="5"/>
@@ -493,6 +570,9 @@
       <x:c r="D23" s="6"/>
       <x:c r="E23" s="5"/>
       <x:c r="F23" s="5"/>
+      <x:c r="G23" s="7"/>
+      <x:c r="H23" s="7"/>
+      <x:c r="I23" s="5"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="5"/>
@@ -501,6 +581,9 @@
       <x:c r="D24" s="6"/>
       <x:c r="E24" s="5"/>
       <x:c r="F24" s="5"/>
+      <x:c r="G24" s="7"/>
+      <x:c r="H24" s="7"/>
+      <x:c r="I24" s="5"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="5"/>
@@ -509,6 +592,9 @@
       <x:c r="D25" s="6"/>
       <x:c r="E25" s="5"/>
       <x:c r="F25" s="5"/>
+      <x:c r="G25" s="7"/>
+      <x:c r="H25" s="7"/>
+      <x:c r="I25" s="5"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="5"/>
@@ -517,6 +603,9 @@
       <x:c r="D26" s="6"/>
       <x:c r="E26" s="5"/>
       <x:c r="F26" s="5"/>
+      <x:c r="G26" s="7"/>
+      <x:c r="H26" s="7"/>
+      <x:c r="I26" s="5"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="5"/>
@@ -525,6 +614,9 @@
       <x:c r="D27" s="6"/>
       <x:c r="E27" s="5"/>
       <x:c r="F27" s="5"/>
+      <x:c r="G27" s="7"/>
+      <x:c r="H27" s="7"/>
+      <x:c r="I27" s="5"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="5"/>
@@ -533,6 +625,9 @@
       <x:c r="D28" s="6"/>
       <x:c r="E28" s="5"/>
       <x:c r="F28" s="5"/>
+      <x:c r="G28" s="7"/>
+      <x:c r="H28" s="7"/>
+      <x:c r="I28" s="5"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="5"/>
@@ -541,6 +636,9 @@
       <x:c r="D29" s="6"/>
       <x:c r="E29" s="5"/>
       <x:c r="F29" s="5"/>
+      <x:c r="G29" s="7"/>
+      <x:c r="H29" s="7"/>
+      <x:c r="I29" s="5"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="5"/>
@@ -549,6 +647,9 @@
       <x:c r="D30" s="6"/>
       <x:c r="E30" s="5"/>
       <x:c r="F30" s="5"/>
+      <x:c r="G30" s="7"/>
+      <x:c r="H30" s="7"/>
+      <x:c r="I30" s="5"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="5"/>
@@ -557,6 +658,9 @@
       <x:c r="D31" s="6"/>
       <x:c r="E31" s="5"/>
       <x:c r="F31" s="5"/>
+      <x:c r="G31" s="7"/>
+      <x:c r="H31" s="7"/>
+      <x:c r="I31" s="5"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="5"/>
@@ -565,6 +669,9 @@
       <x:c r="D32" s="6"/>
       <x:c r="E32" s="5"/>
       <x:c r="F32" s="5"/>
+      <x:c r="G32" s="7"/>
+      <x:c r="H32" s="7"/>
+      <x:c r="I32" s="5"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="5"/>
@@ -573,6 +680,9 @@
       <x:c r="D33" s="6"/>
       <x:c r="E33" s="5"/>
       <x:c r="F33" s="5"/>
+      <x:c r="G33" s="7"/>
+      <x:c r="H33" s="7"/>
+      <x:c r="I33" s="5"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="5"/>
@@ -581,6 +691,9 @@
       <x:c r="D34" s="6"/>
       <x:c r="E34" s="5"/>
       <x:c r="F34" s="5"/>
+      <x:c r="G34" s="7"/>
+      <x:c r="H34" s="7"/>
+      <x:c r="I34" s="5"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="5"/>
@@ -589,6 +702,9 @@
       <x:c r="D35" s="6"/>
       <x:c r="E35" s="5"/>
       <x:c r="F35" s="5"/>
+      <x:c r="G35" s="7"/>
+      <x:c r="H35" s="7"/>
+      <x:c r="I35" s="5"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="5"/>
@@ -597,6 +713,9 @@
       <x:c r="D36" s="6"/>
       <x:c r="E36" s="5"/>
       <x:c r="F36" s="5"/>
+      <x:c r="G36" s="7"/>
+      <x:c r="H36" s="7"/>
+      <x:c r="I36" s="5"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="5"/>
@@ -605,6 +724,9 @@
       <x:c r="D37" s="6"/>
       <x:c r="E37" s="5"/>
       <x:c r="F37" s="5"/>
+      <x:c r="G37" s="7"/>
+      <x:c r="H37" s="7"/>
+      <x:c r="I37" s="5"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="5"/>
@@ -613,6 +735,9 @@
       <x:c r="D38" s="6"/>
       <x:c r="E38" s="5"/>
       <x:c r="F38" s="5"/>
+      <x:c r="G38" s="7"/>
+      <x:c r="H38" s="7"/>
+      <x:c r="I38" s="5"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="5"/>
@@ -621,6 +746,9 @@
       <x:c r="D39" s="6"/>
       <x:c r="E39" s="5"/>
       <x:c r="F39" s="5"/>
+      <x:c r="G39" s="7"/>
+      <x:c r="H39" s="7"/>
+      <x:c r="I39" s="5"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="5"/>
@@ -629,6 +757,9 @@
       <x:c r="D40" s="6"/>
       <x:c r="E40" s="5"/>
       <x:c r="F40" s="5"/>
+      <x:c r="G40" s="7"/>
+      <x:c r="H40" s="7"/>
+      <x:c r="I40" s="5"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="5"/>
@@ -637,6 +768,9 @@
       <x:c r="D41" s="6"/>
       <x:c r="E41" s="5"/>
       <x:c r="F41" s="5"/>
+      <x:c r="G41" s="7"/>
+      <x:c r="H41" s="7"/>
+      <x:c r="I41" s="5"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="5"/>
@@ -645,6 +779,9 @@
       <x:c r="D42" s="6"/>
       <x:c r="E42" s="5"/>
       <x:c r="F42" s="5"/>
+      <x:c r="G42" s="7"/>
+      <x:c r="H42" s="7"/>
+      <x:c r="I42" s="5"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="5"/>
@@ -653,6 +790,9 @@
       <x:c r="D43" s="6"/>
       <x:c r="E43" s="5"/>
       <x:c r="F43" s="5"/>
+      <x:c r="G43" s="7"/>
+      <x:c r="H43" s="7"/>
+      <x:c r="I43" s="5"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="5"/>
@@ -661,6 +801,9 @@
       <x:c r="D44" s="6"/>
       <x:c r="E44" s="5"/>
       <x:c r="F44" s="5"/>
+      <x:c r="G44" s="7"/>
+      <x:c r="H44" s="7"/>
+      <x:c r="I44" s="5"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="5"/>
@@ -669,6 +812,9 @@
       <x:c r="D45" s="6"/>
       <x:c r="E45" s="5"/>
       <x:c r="F45" s="5"/>
+      <x:c r="G45" s="7"/>
+      <x:c r="H45" s="7"/>
+      <x:c r="I45" s="5"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="5"/>
@@ -677,6 +823,9 @@
       <x:c r="D46" s="6"/>
       <x:c r="E46" s="5"/>
       <x:c r="F46" s="5"/>
+      <x:c r="G46" s="7"/>
+      <x:c r="H46" s="7"/>
+      <x:c r="I46" s="5"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="5"/>
@@ -685,6 +834,9 @@
       <x:c r="D47" s="6"/>
       <x:c r="E47" s="5"/>
       <x:c r="F47" s="5"/>
+      <x:c r="G47" s="7"/>
+      <x:c r="H47" s="7"/>
+      <x:c r="I47" s="5"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="5"/>
@@ -693,6 +845,9 @@
       <x:c r="D48" s="6"/>
       <x:c r="E48" s="5"/>
       <x:c r="F48" s="5"/>
+      <x:c r="G48" s="7"/>
+      <x:c r="H48" s="7"/>
+      <x:c r="I48" s="5"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="5"/>
@@ -701,6 +856,9 @@
       <x:c r="D49" s="6"/>
       <x:c r="E49" s="5"/>
       <x:c r="F49" s="5"/>
+      <x:c r="G49" s="7"/>
+      <x:c r="H49" s="7"/>
+      <x:c r="I49" s="5"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="5"/>
@@ -709,6 +867,9 @@
       <x:c r="D50" s="6"/>
       <x:c r="E50" s="5"/>
       <x:c r="F50" s="5"/>
+      <x:c r="G50" s="7"/>
+      <x:c r="H50" s="7"/>
+      <x:c r="I50" s="5"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="5"/>
@@ -717,6 +878,9 @@
       <x:c r="D51" s="6"/>
       <x:c r="E51" s="5"/>
       <x:c r="F51" s="5"/>
+      <x:c r="G51" s="7"/>
+      <x:c r="H51" s="7"/>
+      <x:c r="I51" s="5"/>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="5"/>
@@ -725,6 +889,9 @@
       <x:c r="D52" s="6"/>
       <x:c r="E52" s="5"/>
       <x:c r="F52" s="5"/>
+      <x:c r="G52" s="7"/>
+      <x:c r="H52" s="7"/>
+      <x:c r="I52" s="5"/>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="5"/>
@@ -733,6 +900,9 @@
       <x:c r="D53" s="6"/>
       <x:c r="E53" s="5"/>
       <x:c r="F53" s="5"/>
+      <x:c r="G53" s="7"/>
+      <x:c r="H53" s="7"/>
+      <x:c r="I53" s="5"/>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="5"/>
@@ -741,6 +911,9 @@
       <x:c r="D54" s="6"/>
       <x:c r="E54" s="5"/>
       <x:c r="F54" s="5"/>
+      <x:c r="G54" s="7"/>
+      <x:c r="H54" s="7"/>
+      <x:c r="I54" s="5"/>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="5"/>
@@ -749,6 +922,9 @@
       <x:c r="D55" s="6"/>
       <x:c r="E55" s="5"/>
       <x:c r="F55" s="5"/>
+      <x:c r="G55" s="7"/>
+      <x:c r="H55" s="7"/>
+      <x:c r="I55" s="5"/>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="5"/>
@@ -757,6 +933,9 @@
       <x:c r="D56" s="6"/>
       <x:c r="E56" s="5"/>
       <x:c r="F56" s="5"/>
+      <x:c r="G56" s="7"/>
+      <x:c r="H56" s="7"/>
+      <x:c r="I56" s="5"/>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="5"/>
@@ -765,6 +944,9 @@
       <x:c r="D57" s="6"/>
       <x:c r="E57" s="5"/>
       <x:c r="F57" s="5"/>
+      <x:c r="G57" s="7"/>
+      <x:c r="H57" s="7"/>
+      <x:c r="I57" s="5"/>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="5"/>
@@ -773,6 +955,9 @@
       <x:c r="D58" s="6"/>
       <x:c r="E58" s="5"/>
       <x:c r="F58" s="5"/>
+      <x:c r="G58" s="7"/>
+      <x:c r="H58" s="7"/>
+      <x:c r="I58" s="5"/>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="5"/>
@@ -781,6 +966,9 @@
       <x:c r="D59" s="6"/>
       <x:c r="E59" s="5"/>
       <x:c r="F59" s="5"/>
+      <x:c r="G59" s="7"/>
+      <x:c r="H59" s="7"/>
+      <x:c r="I59" s="5"/>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="5"/>
@@ -789,6 +977,9 @@
       <x:c r="D60" s="6"/>
       <x:c r="E60" s="5"/>
       <x:c r="F60" s="5"/>
+      <x:c r="G60" s="7"/>
+      <x:c r="H60" s="7"/>
+      <x:c r="I60" s="5"/>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="5"/>
@@ -797,6 +988,9 @@
       <x:c r="D61" s="6"/>
       <x:c r="E61" s="5"/>
       <x:c r="F61" s="5"/>
+      <x:c r="G61" s="7"/>
+      <x:c r="H61" s="7"/>
+      <x:c r="I61" s="5"/>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="5"/>
@@ -805,6 +999,9 @@
       <x:c r="D62" s="6"/>
       <x:c r="E62" s="5"/>
       <x:c r="F62" s="5"/>
+      <x:c r="G62" s="7"/>
+      <x:c r="H62" s="7"/>
+      <x:c r="I62" s="5"/>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="5"/>
@@ -813,6 +1010,9 @@
       <x:c r="D63" s="6"/>
       <x:c r="E63" s="5"/>
       <x:c r="F63" s="5"/>
+      <x:c r="G63" s="7"/>
+      <x:c r="H63" s="7"/>
+      <x:c r="I63" s="5"/>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="5"/>
@@ -821,6 +1021,9 @@
       <x:c r="D64" s="6"/>
       <x:c r="E64" s="5"/>
       <x:c r="F64" s="5"/>
+      <x:c r="G64" s="7"/>
+      <x:c r="H64" s="7"/>
+      <x:c r="I64" s="5"/>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="5"/>
@@ -829,6 +1032,9 @@
       <x:c r="D65" s="6"/>
       <x:c r="E65" s="5"/>
       <x:c r="F65" s="5"/>
+      <x:c r="G65" s="7"/>
+      <x:c r="H65" s="7"/>
+      <x:c r="I65" s="5"/>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="5"/>
@@ -837,6 +1043,9 @@
       <x:c r="D66" s="6"/>
       <x:c r="E66" s="5"/>
       <x:c r="F66" s="5"/>
+      <x:c r="G66" s="7"/>
+      <x:c r="H66" s="7"/>
+      <x:c r="I66" s="5"/>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="5"/>
@@ -845,6 +1054,9 @@
       <x:c r="D67" s="6"/>
       <x:c r="E67" s="5"/>
       <x:c r="F67" s="5"/>
+      <x:c r="G67" s="7"/>
+      <x:c r="H67" s="7"/>
+      <x:c r="I67" s="5"/>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="5"/>
@@ -853,6 +1065,9 @@
       <x:c r="D68" s="6"/>
       <x:c r="E68" s="5"/>
       <x:c r="F68" s="5"/>
+      <x:c r="G68" s="7"/>
+      <x:c r="H68" s="7"/>
+      <x:c r="I68" s="5"/>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="5"/>
@@ -861,6 +1076,9 @@
       <x:c r="D69" s="6"/>
       <x:c r="E69" s="5"/>
       <x:c r="F69" s="5"/>
+      <x:c r="G69" s="7"/>
+      <x:c r="H69" s="7"/>
+      <x:c r="I69" s="5"/>
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="5"/>
@@ -869,6 +1087,9 @@
       <x:c r="D70" s="6"/>
       <x:c r="E70" s="5"/>
       <x:c r="F70" s="5"/>
+      <x:c r="G70" s="7"/>
+      <x:c r="H70" s="7"/>
+      <x:c r="I70" s="5"/>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="5"/>
@@ -877,6 +1098,9 @@
       <x:c r="D71" s="6"/>
       <x:c r="E71" s="5"/>
       <x:c r="F71" s="5"/>
+      <x:c r="G71" s="7"/>
+      <x:c r="H71" s="7"/>
+      <x:c r="I71" s="5"/>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="5"/>
@@ -885,6 +1109,9 @@
       <x:c r="D72" s="6"/>
       <x:c r="E72" s="5"/>
       <x:c r="F72" s="5"/>
+      <x:c r="G72" s="7"/>
+      <x:c r="H72" s="7"/>
+      <x:c r="I72" s="5"/>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="5"/>
@@ -893,6 +1120,9 @@
       <x:c r="D73" s="6"/>
       <x:c r="E73" s="5"/>
       <x:c r="F73" s="5"/>
+      <x:c r="G73" s="7"/>
+      <x:c r="H73" s="7"/>
+      <x:c r="I73" s="5"/>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="5"/>
@@ -901,6 +1131,9 @@
       <x:c r="D74" s="6"/>
       <x:c r="E74" s="5"/>
       <x:c r="F74" s="5"/>
+      <x:c r="G74" s="7"/>
+      <x:c r="H74" s="7"/>
+      <x:c r="I74" s="5"/>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="5"/>
@@ -909,6 +1142,9 @@
       <x:c r="D75" s="6"/>
       <x:c r="E75" s="5"/>
       <x:c r="F75" s="5"/>
+      <x:c r="G75" s="7"/>
+      <x:c r="H75" s="7"/>
+      <x:c r="I75" s="5"/>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="5"/>
@@ -917,6 +1153,9 @@
       <x:c r="D76" s="6"/>
       <x:c r="E76" s="5"/>
       <x:c r="F76" s="5"/>
+      <x:c r="G76" s="7"/>
+      <x:c r="H76" s="7"/>
+      <x:c r="I76" s="5"/>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="5"/>
@@ -925,6 +1164,9 @@
       <x:c r="D77" s="6"/>
       <x:c r="E77" s="5"/>
       <x:c r="F77" s="5"/>
+      <x:c r="G77" s="7"/>
+      <x:c r="H77" s="7"/>
+      <x:c r="I77" s="5"/>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="5"/>
@@ -933,6 +1175,9 @@
       <x:c r="D78" s="6"/>
       <x:c r="E78" s="5"/>
       <x:c r="F78" s="5"/>
+      <x:c r="G78" s="7"/>
+      <x:c r="H78" s="7"/>
+      <x:c r="I78" s="5"/>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="5"/>
@@ -941,6 +1186,9 @@
       <x:c r="D79" s="6"/>
       <x:c r="E79" s="5"/>
       <x:c r="F79" s="5"/>
+      <x:c r="G79" s="7"/>
+      <x:c r="H79" s="7"/>
+      <x:c r="I79" s="5"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="5"/>
@@ -949,6 +1197,9 @@
       <x:c r="D80" s="6"/>
       <x:c r="E80" s="5"/>
       <x:c r="F80" s="5"/>
+      <x:c r="G80" s="7"/>
+      <x:c r="H80" s="7"/>
+      <x:c r="I80" s="5"/>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="5"/>
@@ -957,6 +1208,9 @@
       <x:c r="D81" s="6"/>
       <x:c r="E81" s="5"/>
       <x:c r="F81" s="5"/>
+      <x:c r="G81" s="7"/>
+      <x:c r="H81" s="7"/>
+      <x:c r="I81" s="5"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="5"/>
@@ -965,6 +1219,9 @@
       <x:c r="D82" s="6"/>
       <x:c r="E82" s="5"/>
       <x:c r="F82" s="5"/>
+      <x:c r="G82" s="7"/>
+      <x:c r="H82" s="7"/>
+      <x:c r="I82" s="5"/>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="5"/>
@@ -973,6 +1230,9 @@
       <x:c r="D83" s="6"/>
       <x:c r="E83" s="5"/>
       <x:c r="F83" s="5"/>
+      <x:c r="G83" s="7"/>
+      <x:c r="H83" s="7"/>
+      <x:c r="I83" s="5"/>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="5"/>
@@ -981,6 +1241,9 @@
       <x:c r="D84" s="6"/>
       <x:c r="E84" s="5"/>
       <x:c r="F84" s="5"/>
+      <x:c r="G84" s="7"/>
+      <x:c r="H84" s="7"/>
+      <x:c r="I84" s="5"/>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="5"/>
@@ -989,6 +1252,9 @@
       <x:c r="D85" s="6"/>
       <x:c r="E85" s="5"/>
       <x:c r="F85" s="5"/>
+      <x:c r="G85" s="7"/>
+      <x:c r="H85" s="7"/>
+      <x:c r="I85" s="5"/>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="5"/>
@@ -997,6 +1263,9 @@
       <x:c r="D86" s="6"/>
       <x:c r="E86" s="5"/>
       <x:c r="F86" s="5"/>
+      <x:c r="G86" s="7"/>
+      <x:c r="H86" s="7"/>
+      <x:c r="I86" s="5"/>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="5"/>
@@ -1005,6 +1274,9 @@
       <x:c r="D87" s="6"/>
       <x:c r="E87" s="5"/>
       <x:c r="F87" s="5"/>
+      <x:c r="G87" s="7"/>
+      <x:c r="H87" s="7"/>
+      <x:c r="I87" s="5"/>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="5"/>
@@ -1013,6 +1285,9 @@
       <x:c r="D88" s="6"/>
       <x:c r="E88" s="5"/>
       <x:c r="F88" s="5"/>
+      <x:c r="G88" s="7"/>
+      <x:c r="H88" s="7"/>
+      <x:c r="I88" s="5"/>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="5"/>
@@ -1021,6 +1296,9 @@
       <x:c r="D89" s="6"/>
       <x:c r="E89" s="5"/>
       <x:c r="F89" s="5"/>
+      <x:c r="G89" s="7"/>
+      <x:c r="H89" s="7"/>
+      <x:c r="I89" s="5"/>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="5"/>
@@ -1029,6 +1307,9 @@
       <x:c r="D90" s="6"/>
       <x:c r="E90" s="5"/>
       <x:c r="F90" s="5"/>
+      <x:c r="G90" s="7"/>
+      <x:c r="H90" s="7"/>
+      <x:c r="I90" s="5"/>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="5"/>
@@ -1037,6 +1318,9 @@
       <x:c r="D91" s="6"/>
       <x:c r="E91" s="5"/>
       <x:c r="F91" s="5"/>
+      <x:c r="G91" s="7"/>
+      <x:c r="H91" s="7"/>
+      <x:c r="I91" s="5"/>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="5"/>
@@ -1045,6 +1329,9 @@
       <x:c r="D92" s="6"/>
       <x:c r="E92" s="5"/>
       <x:c r="F92" s="5"/>
+      <x:c r="G92" s="7"/>
+      <x:c r="H92" s="7"/>
+      <x:c r="I92" s="5"/>
     </x:row>
     <x:row r="93" ht="23" customHeight="1">
       <x:c r="A93" s="5"/>
@@ -1053,6 +1340,9 @@
       <x:c r="D93" s="6"/>
       <x:c r="E93" s="5"/>
       <x:c r="F93" s="5"/>
+      <x:c r="G93" s="7"/>
+      <x:c r="H93" s="7"/>
+      <x:c r="I93" s="5"/>
     </x:row>
     <x:row r="94" ht="23" customHeight="1">
       <x:c r="A94" s="5"/>
@@ -1061,6 +1351,9 @@
       <x:c r="D94" s="6"/>
       <x:c r="E94" s="5"/>
       <x:c r="F94" s="5"/>
+      <x:c r="G94" s="7"/>
+      <x:c r="H94" s="7"/>
+      <x:c r="I94" s="5"/>
     </x:row>
     <x:row r="95" ht="23" customHeight="1">
       <x:c r="A95" s="5"/>
@@ -1069,6 +1362,9 @@
       <x:c r="D95" s="6"/>
       <x:c r="E95" s="5"/>
       <x:c r="F95" s="5"/>
+      <x:c r="G95" s="7"/>
+      <x:c r="H95" s="7"/>
+      <x:c r="I95" s="5"/>
     </x:row>
     <x:row r="96" ht="23" customHeight="1">
       <x:c r="A96" s="5"/>
@@ -1077,6 +1373,9 @@
       <x:c r="D96" s="6"/>
       <x:c r="E96" s="5"/>
       <x:c r="F96" s="5"/>
+      <x:c r="G96" s="7"/>
+      <x:c r="H96" s="7"/>
+      <x:c r="I96" s="5"/>
     </x:row>
     <x:row r="97" ht="23" customHeight="1">
       <x:c r="A97" s="5"/>
@@ -1085,6 +1384,9 @@
       <x:c r="D97" s="6"/>
       <x:c r="E97" s="5"/>
       <x:c r="F97" s="5"/>
+      <x:c r="G97" s="7"/>
+      <x:c r="H97" s="7"/>
+      <x:c r="I97" s="5"/>
     </x:row>
     <x:row r="98" ht="23" customHeight="1">
       <x:c r="A98" s="5"/>
@@ -1093,6 +1395,9 @@
       <x:c r="D98" s="6"/>
       <x:c r="E98" s="5"/>
       <x:c r="F98" s="5"/>
+      <x:c r="G98" s="7"/>
+      <x:c r="H98" s="7"/>
+      <x:c r="I98" s="5"/>
     </x:row>
     <x:row r="99" ht="23" customHeight="1">
       <x:c r="A99" s="5"/>
@@ -1101,6 +1406,9 @@
       <x:c r="D99" s="6"/>
       <x:c r="E99" s="5"/>
       <x:c r="F99" s="5"/>
+      <x:c r="G99" s="7"/>
+      <x:c r="H99" s="7"/>
+      <x:c r="I99" s="5"/>
     </x:row>
     <x:row r="100" ht="23" customHeight="1">
       <x:c r="A100" s="5"/>
@@ -1109,6 +1417,9 @@
       <x:c r="D100" s="6"/>
       <x:c r="E100" s="5"/>
       <x:c r="F100" s="5"/>
+      <x:c r="G100" s="7"/>
+      <x:c r="H100" s="7"/>
+      <x:c r="I100" s="5"/>
     </x:row>
     <x:row r="101" ht="23" customHeight="1">
       <x:c r="A101" s="5"/>
@@ -1117,9 +1428,15 @@
       <x:c r="D101" s="6"/>
       <x:c r="E101" s="5"/>
       <x:c r="F101" s="5"/>
+      <x:c r="G101" s="7"/>
+      <x:c r="H101" s="7"/>
+      <x:c r="I101" s="5"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="I2:I101">
+      <x:formula1>"fixed,m2,v2"</x:formula1>
+    </x:dataValidation>
     <x:dataValidation type="list" sqref="E2:E101">
       <x:formula1>"HNL,USD"</x:formula1>
     </x:dataValidation>
@@ -1137,7 +1454,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="2">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="A2" s="8" t="str">
         <x:v>Plantilla de lotes</x:v>
       </x:c>
     </x:row>
@@ -1158,36 +1475,46 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>Precio: importe con máximo dos decimales, sin símbolo monetario.</x:v>
+        <x:v>Área: complete m² o vara², hasta seis decimales. Si llena ambas, deben coincidir.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="1" t="str">
-        <x:v>Moneda: HNL o USD.</x:v>
+        <x:v>Unidad de precio: fixed (precio fijo), m2 o v2. Las tarifas se configuran en el sistema.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="1" t="str">
-        <x:v>Estado: deje vacío para nuevos lotes. Disponible, Reservado o Vendido solo puede conservar el estado actual.</x:v>
+        <x:v>Precio: importe con máximo dos decimales, sin símbolo monetario.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="1" t="str">
-        <x:v>El estado lo determinan las reservas y contratos. No se cambian ventas previas al editar el precio base.</x:v>
+        <x:v>Moneda: HNL o USD.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="1" t="str">
-        <x:v>Crear y actualizar identifica por ID o por código.</x:v>
+        <x:v>Estado: deje vacío para nuevos lotes. Disponible, Reservado o Vendido solo puede conservar el estado actual.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="1" t="str">
-        <x:v>No use fórmulas. Se admite un máximo de 10,000 registros por archivo.</x:v>
+        <x:v>El estado lo determinan las reservas y contratos. No se cambian ventas previas al editar el precio base.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="1" t="str">
+        <x:v>Crear y actualizar identifica por ID o por código.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="25" customHeight="1">
+      <x:c r="A14" s="1" t="str">
+        <x:v>No use fórmulas. Se admite un máximo de 10,000 registros por archivo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="A15" s="1" t="str">
         <x:v>El ejemplo de esta hoja es ficticio y no se importa. La hoja de datos está vacía.</x:v>
       </x:c>
     </x:row>
@@ -1197,32 +1524,38 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="8" t="str">
+      <x:c r="A17" s="9" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B17" s="9" t="str"/>
-      <x:c r="C17" s="8"/>
-      <x:c r="D17" s="8"/>
-      <x:c r="E17" s="8"/>
-      <x:c r="F17" s="8"/>
+      <x:c r="B17" s="10" t="str"/>
+      <x:c r="C17" s="9"/>
+      <x:c r="D17" s="9"/>
+      <x:c r="E17" s="9"/>
+      <x:c r="F17" s="9"/>
+      <x:c r="G17" s="9"/>
+      <x:c r="H17" s="9"/>
+      <x:c r="I17" s="9"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="str">
         <x:v>Código</x:v>
       </x:c>
-      <x:c r="B18" s="10" t="str">
+      <x:c r="B18" s="11" t="str">
         <x:v>RP-001</x:v>
       </x:c>
       <x:c r="C18" s="1"/>
       <x:c r="D18" s="1"/>
       <x:c r="E18" s="1"/>
       <x:c r="F18" s="1"/>
+      <x:c r="G18" s="1"/>
+      <x:c r="H18" s="1"/>
+      <x:c r="I18" s="1"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
         <x:v>Descripción</x:v>
       </x:c>
-      <x:c r="B19" s="11" t="str">
+      <x:c r="B19" s="12" t="str">
         <x:v>Manzana A</x:v>
       </x:c>
     </x:row>
@@ -1230,7 +1563,7 @@
       <x:c r="A20" t="str">
         <x:v>Precio</x:v>
       </x:c>
-      <x:c r="B20" s="12" t="n">
+      <x:c r="B20" s="13" t="n">
         <x:v>200000</x:v>
       </x:c>
     </x:row>
@@ -1238,7 +1571,7 @@
       <x:c r="A21" t="str">
         <x:v>Moneda</x:v>
       </x:c>
-      <x:c r="B21" s="11" t="str">
+      <x:c r="B21" s="12" t="str">
         <x:v>HNL</x:v>
       </x:c>
     </x:row>
@@ -1246,7 +1579,29 @@
       <x:c r="A22" t="str">
         <x:v>Estado</x:v>
       </x:c>
-      <x:c r="B22" s="11" t="str"/>
+      <x:c r="B22" s="12" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Área m²</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="n">
+        <x:v>116.25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>Área vara²</x:v>
+      </x:c>
+      <x:c r="B24" s="12" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>Unidad de precio</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="str">
+        <x:v>m2</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>